<commit_message>
Deploying to gh-pages from @ pchelle/OSPSuite.ReportingEngine@252a1667c9e5c8ee8ce6d30702646d25f1ab6f45 🚀
</commit_message>
<xml_diff>
--- a/docs/dev/articles/templates/WorkflowInput.xlsx
+++ b/docs/dev/articles/templates/WorkflowInput.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Design2Code\OSPSuite.ReportingEngine\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pierre Chelle\Documents\Design2Code\OSPSuite.ReportingEngine\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6244981-9F1B-4280-9D87-79CDA783064A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{837E7BE3-612B-4C2C-885D-28F9B403B082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="914" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="914" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Documentation" sheetId="12" r:id="rId1"/>
@@ -25,15 +25,16 @@
     <sheet name="PK Fraction" sheetId="19" r:id="rId10"/>
     <sheet name="SensitivityParameter" sheetId="7" r:id="rId11"/>
     <sheet name="tpDictionary" sheetId="11" r:id="rId12"/>
-    <sheet name="StudyDesign" sheetId="21" r:id="rId13"/>
-    <sheet name="Lookup" sheetId="16" r:id="rId14"/>
+    <sheet name="tpDictionaryLoq" sheetId="23" r:id="rId13"/>
+    <sheet name="StudyDesign" sheetId="21" r:id="rId14"/>
+    <sheet name="Lookup" sheetId="16" r:id="rId15"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="418">
   <si>
     <t>reportName</t>
   </si>
@@ -1889,7 +1890,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1959,6 +1960,8 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2496,12 +2499,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.125" customWidth="1"/>
+    <col min="1" max="1" width="20.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>93</v>
       </c>
@@ -2509,7 +2512,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>94</v>
       </c>
@@ -2517,7 +2520,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>95</v>
       </c>
@@ -2534,13 +2537,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>158</v>
       </c>
@@ -2551,12 +2554,12 @@
         <v>159</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -2570,22 +2573,22 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="61" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>317</v>
       </c>
@@ -2598,15 +2601,15 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="13.5" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
-    <col min="7" max="7" width="48.125" customWidth="1"/>
+    <col min="7" max="7" width="48.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>318</v>
       </c>
@@ -2629,7 +2632,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>54</v>
       </c>
@@ -2644,7 +2647,7 @@
       <c r="F2" s="9"/>
       <c r="G2" s="9"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>57</v>
       </c>
@@ -2659,7 +2662,7 @@
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>59</v>
       </c>
@@ -2676,7 +2679,7 @@
       <c r="F4" s="9"/>
       <c r="G4" s="9"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>62</v>
       </c>
@@ -2693,7 +2696,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>65</v>
       </c>
@@ -2710,7 +2713,7 @@
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>69</v>
       </c>
@@ -2731,7 +2734,7 @@
       </c>
       <c r="G7" s="9"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>75</v>
       </c>
@@ -2752,7 +2755,7 @@
       </c>
       <c r="G8" s="9"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>80</v>
       </c>
@@ -2773,7 +2776,7 @@
       </c>
       <c r="G9" s="9"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>85</v>
       </c>
@@ -2794,7 +2797,7 @@
       </c>
       <c r="G10" s="9"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>89</v>
       </c>
@@ -2813,23 +2816,6 @@
       </c>
       <c r="G11" s="9" t="s">
         <v>417</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2839,17 +2825,262 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05B762A-0A3E-4AE3-9238-C14EE5C34AFE}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.58203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="42.4140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="31" t="s">
+        <v>318</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="31" t="s">
+        <v>412</v>
+      </c>
+      <c r="D1" s="31" t="s">
+        <v>413</v>
+      </c>
+      <c r="E1" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="32" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="32"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="32"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" s="32"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="G10" s="32"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="32" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.375" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
     <col min="2" max="2" width="18.25" customWidth="1"/>
-    <col min="3" max="3" width="19.125" customWidth="1"/>
+    <col min="3" max="3" width="19.08203125" customWidth="1"/>
     <col min="4" max="4" width="40.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>79</v>
       </c>
@@ -2863,7 +3094,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>77</v>
       </c>
@@ -2875,7 +3106,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>354</v>
       </c>
@@ -2889,7 +3120,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
         <v>20</v>
       </c>
@@ -2903,7 +3134,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>20</v>
       </c>
@@ -2917,7 +3148,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
         <v>40</v>
       </c>
@@ -2931,7 +3162,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
         <v>40</v>
       </c>
@@ -2945,7 +3176,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
         <v>60</v>
       </c>
@@ -2961,24 +3192,24 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:M37"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.58203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.08203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="10" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>103</v>
       </c>
@@ -3019,7 +3250,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>105</v>
       </c>
@@ -3060,7 +3291,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>104</v>
       </c>
@@ -3101,7 +3332,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>107</v>
       </c>
@@ -3127,7 +3358,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E5" t="s">
         <v>162</v>
       </c>
@@ -3150,7 +3381,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>163</v>
       </c>
@@ -3170,7 +3401,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
         <v>164</v>
       </c>
@@ -3190,7 +3421,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
         <v>165</v>
       </c>
@@ -3210,7 +3441,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
         <v>166</v>
       </c>
@@ -3230,7 +3461,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
         <v>167</v>
       </c>
@@ -3244,7 +3475,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
         <v>168</v>
       </c>
@@ -3258,7 +3489,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>169</v>
       </c>
@@ -3272,7 +3503,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E13" t="s">
         <v>170</v>
       </c>
@@ -3286,7 +3517,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E14" t="s">
         <v>171</v>
       </c>
@@ -3300,7 +3531,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E15" t="s">
         <v>172</v>
       </c>
@@ -3314,7 +3545,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="E16" t="s">
         <v>173</v>
       </c>
@@ -3328,7 +3559,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="17" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E17" t="s">
         <v>174</v>
       </c>
@@ -3342,7 +3573,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="18" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="18" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E18" t="s">
         <v>175</v>
       </c>
@@ -3356,7 +3587,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="19" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E19" t="s">
         <v>176</v>
       </c>
@@ -3370,7 +3601,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="20" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E20" t="s">
         <v>177</v>
       </c>
@@ -3384,7 +3615,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="21" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E21" t="s">
         <v>178</v>
       </c>
@@ -3398,7 +3629,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="22" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E22" t="s">
         <v>179</v>
       </c>
@@ -3412,7 +3643,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="23" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E23" t="s">
         <v>180</v>
       </c>
@@ -3420,7 +3651,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="24" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E24" t="s">
         <v>181</v>
       </c>
@@ -3428,7 +3659,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="25" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E25" t="s">
         <v>182</v>
       </c>
@@ -3436,7 +3667,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="26" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E26" t="s">
         <v>183</v>
       </c>
@@ -3444,7 +3675,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="27" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E27" t="s">
         <v>184</v>
       </c>
@@ -3452,7 +3683,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="28" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E28" t="s">
         <v>185</v>
       </c>
@@ -3460,7 +3691,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="29" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E29" t="s">
         <v>186</v>
       </c>
@@ -3468,42 +3699,42 @@
         <v>227</v>
       </c>
     </row>
-    <row r="30" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="5:13" x14ac:dyDescent="0.3">
       <c r="G30" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="31" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="5:13" x14ac:dyDescent="0.3">
       <c r="G31" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="32" spans="5:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="5:13" x14ac:dyDescent="0.3">
       <c r="G32" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="33" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G33" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="34" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G34" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G35" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="36" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G36" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="37" spans="7:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="7:7" x14ac:dyDescent="0.3">
       <c r="G37" t="s">
         <v>234</v>
       </c>
@@ -3517,7 +3748,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="100.25" customWidth="1"/>
@@ -3525,7 +3756,7 @@
     <col min="6" max="6" width="22.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>1</v>
       </c>
@@ -3536,7 +3767,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="38" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>100</v>
       </c>
@@ -3547,7 +3778,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>101</v>
       </c>
@@ -3558,7 +3789,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
         <v>129</v>
       </c>
@@ -3569,7 +3800,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
         <v>378</v>
       </c>
@@ -3578,7 +3809,7 @@
       </c>
       <c r="C5" s="15"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
         <v>331</v>
       </c>
@@ -3587,7 +3818,7 @@
       </c>
       <c r="C6" s="15"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
         <v>131</v>
       </c>
@@ -3598,7 +3829,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
         <v>365</v>
       </c>
@@ -3607,7 +3838,7 @@
       </c>
       <c r="C8" s="15"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
         <v>320</v>
       </c>
@@ -3616,14 +3847,14 @@
       </c>
       <c r="C9" s="15"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="28" t="s">
         <v>329</v>
       </c>
       <c r="B10" s="28"/>
       <c r="C10" s="28"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>111</v>
       </c>
@@ -3634,7 +3865,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
         <v>113</v>
       </c>
@@ -3645,7 +3876,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
         <v>115</v>
       </c>
@@ -3656,7 +3887,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
         <v>117</v>
       </c>
@@ -3667,7 +3898,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
         <v>119</v>
       </c>
@@ -3678,7 +3909,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
         <v>121</v>
       </c>
@@ -3689,7 +3920,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
         <v>123</v>
       </c>
@@ -3700,7 +3931,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
         <v>124</v>
       </c>
@@ -3711,7 +3942,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
         <v>125</v>
       </c>
@@ -3722,14 +3953,14 @@
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="28" t="s">
         <v>330</v>
       </c>
       <c r="B20" s="28"/>
       <c r="C20" s="28"/>
     </row>
-    <row r="21" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="38.5" x14ac:dyDescent="0.3">
       <c r="A21" s="14" t="s">
         <v>132</v>
       </c>
@@ -3738,7 +3969,7 @@
       </c>
       <c r="C21" s="15"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
         <v>133</v>
       </c>
@@ -3749,7 +3980,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="51" x14ac:dyDescent="0.3">
       <c r="A23" s="14" t="s">
         <v>137</v>
       </c>
@@ -3758,7 +3989,7 @@
       </c>
       <c r="C23" s="15"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
         <v>138</v>
       </c>
@@ -3767,7 +3998,7 @@
       </c>
       <c r="C24" s="15"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
         <v>140</v>
       </c>
@@ -3778,7 +4009,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="14" t="s">
         <v>141</v>
       </c>
@@ -3787,7 +4018,7 @@
       </c>
       <c r="C26" s="15"/>
     </row>
-    <row r="27" spans="1:3" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="38" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
         <v>155</v>
       </c>
@@ -3796,7 +4027,7 @@
       </c>
       <c r="C27" s="15"/>
     </row>
-    <row r="28" spans="1:3" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
         <v>147</v>
       </c>
@@ -3805,7 +4036,7 @@
       </c>
       <c r="C28" s="15"/>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="14" t="s">
         <v>148</v>
       </c>
@@ -3814,7 +4045,7 @@
       </c>
       <c r="C29" s="15"/>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
         <v>151</v>
       </c>
@@ -3823,7 +4054,7 @@
       </c>
       <c r="C30" s="15"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>153</v>
       </c>
@@ -3832,14 +4063,14 @@
       </c>
       <c r="C31" s="15"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="28" t="s">
         <v>349</v>
       </c>
       <c r="B32" s="28"/>
       <c r="C32" s="28"/>
     </row>
-    <row r="33" spans="1:3" ht="51.75" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" ht="51" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
         <v>350</v>
       </c>
@@ -3940,15 +4171,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.875" customWidth="1"/>
-    <col min="2" max="2" width="42.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.75" customWidth="1"/>
     <col min="4" max="4" width="29.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="18" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>1</v>
       </c>
@@ -3962,7 +4193,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>291</v>
       </c>
@@ -3970,7 +4201,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="18" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" s="18" customFormat="1" ht="38.5" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>293</v>
       </c>
@@ -3978,7 +4209,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="18" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" s="18" customFormat="1" ht="38.5" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>4</v>
       </c>
@@ -3992,7 +4223,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="18" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" s="18" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>381</v>
       </c>
@@ -4000,7 +4231,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="18" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" s="18" customFormat="1" ht="75.5" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>285</v>
       </c>
@@ -4014,7 +4245,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="18" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" s="18" customFormat="1" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
         <v>286</v>
       </c>
@@ -4028,7 +4259,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
         <v>303</v>
       </c>
@@ -4042,7 +4273,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>322</v>
       </c>
@@ -4056,7 +4287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
         <v>305</v>
       </c>
@@ -4064,7 +4295,7 @@
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
     </row>
-    <row r="11" spans="1:4" s="18" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" s="18" customFormat="1" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>306</v>
       </c>
@@ -4072,7 +4303,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>308</v>
       </c>
@@ -4080,7 +4311,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="18" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" s="18" customFormat="1" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
         <v>310</v>
       </c>
@@ -4094,7 +4325,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:4" s="18" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" s="18" customFormat="1" ht="38" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
         <v>324</v>
       </c>
@@ -4108,7 +4339,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="15" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
         <v>311</v>
       </c>
@@ -4122,7 +4353,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="16" spans="1:4" s="18" customFormat="1" ht="89.25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" s="18" customFormat="1" ht="89" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
         <v>312</v>
       </c>
@@ -4133,7 +4364,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="29" t="s">
         <v>414</v>
       </c>
@@ -4141,7 +4372,7 @@
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
     </row>
-    <row r="18" spans="1:4" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="38" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>415</v>
       </c>
@@ -4211,15 +4442,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.75" style="6" customWidth="1"/>
-    <col min="2" max="2" width="30.625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="47.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.58203125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="47.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="23" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>1</v>
       </c>
@@ -4233,7 +4464,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>283</v>
       </c>
@@ -4247,7 +4478,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>284</v>
       </c>
@@ -4261,7 +4492,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>11</v>
       </c>
@@ -4275,7 +4506,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="18" customFormat="1" ht="57" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" s="18" customFormat="1" ht="56" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>376</v>
       </c>
@@ -4283,7 +4514,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="18" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" s="18" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>383</v>
       </c>
@@ -4294,7 +4525,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="18" customFormat="1" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" s="18" customFormat="1" ht="42" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
         <v>384</v>
       </c>
@@ -4305,7 +4536,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="18" customFormat="1" ht="142.5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" s="18" customFormat="1" ht="140" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
         <v>285</v>
       </c>
@@ -4319,7 +4550,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="18" customFormat="1" ht="57" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" s="18" customFormat="1" ht="56" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>286</v>
       </c>
@@ -4333,7 +4564,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="18" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" s="18" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
         <v>367</v>
       </c>
@@ -4342,7 +4573,7 @@
       </c>
       <c r="C10" s="21"/>
     </row>
-    <row r="11" spans="1:4" s="18" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" s="18" customFormat="1" ht="28" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>287</v>
       </c>
@@ -4447,15 +4678,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.375" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="18.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>1</v>
       </c>
@@ -4469,7 +4700,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>371</v>
       </c>
@@ -4479,7 +4710,7 @@
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
     </row>
-    <row r="3" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="25.5" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>300</v>
       </c>
@@ -4493,7 +4724,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="132" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="132" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>296</v>
       </c>
@@ -4505,7 +4736,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="63.5" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>372</v>
       </c>
@@ -4541,21 +4772,21 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.625" customWidth="1"/>
-    <col min="2" max="2" width="27.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.375" customWidth="1"/>
-    <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.58203125" customWidth="1"/>
+    <col min="2" max="2" width="27.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.75" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.75" customWidth="1"/>
-    <col min="8" max="8" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.08203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.5" customWidth="1"/>
     <col min="10" max="10" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.875" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="28" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>158</v>
       </c>
@@ -4592,7 +4823,7 @@
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -4603,7 +4834,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -4643,13 +4874,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>158</v>
       </c>
@@ -4660,7 +4891,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
@@ -4671,7 +4902,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -4682,7 +4913,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -4693,7 +4924,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -4704,7 +4935,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>200</v>
       </c>
@@ -4715,7 +4946,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>235</v>
       </c>
@@ -4726,7 +4957,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
@@ -4737,7 +4968,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
@@ -4748,7 +4979,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
@@ -4759,7 +4990,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
@@ -4770,7 +5001,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -4781,7 +5012,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
@@ -4792,7 +5023,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -4803,7 +5034,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>247</v>
       </c>
@@ -4814,7 +5045,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>248</v>
       </c>
@@ -4825,7 +5056,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>249</v>
       </c>
@@ -4836,7 +5067,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>250</v>
       </c>
@@ -4847,7 +5078,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>251</v>
       </c>
@@ -4858,7 +5089,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>252</v>
       </c>
@@ -4869,7 +5100,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>253</v>
       </c>
@@ -4880,7 +5111,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>254</v>
       </c>
@@ -4891,7 +5122,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>255</v>
       </c>
@@ -4902,7 +5133,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>256</v>
       </c>
@@ -4913,7 +5144,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>257</v>
       </c>
@@ -4924,7 +5155,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>258</v>
       </c>
@@ -4935,7 +5166,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>259</v>
       </c>
@@ -4946,7 +5177,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>260</v>
       </c>
@@ -4957,7 +5188,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>261</v>
       </c>
@@ -4968,7 +5199,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>262</v>
       </c>
@@ -4979,7 +5210,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="31" spans="1:3" s="11" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" s="11" customFormat="1" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="12" t="s">
         <v>263</v>
       </c>
@@ -4990,7 +5221,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" ht="14.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -5001,7 +5232,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -5057,13 +5288,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>158</v>
       </c>
@@ -5074,67 +5305,67 @@
         <v>159</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -5184,13 +5415,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>158</v>
       </c>
@@ -5201,112 +5432,112 @@
         <v>159</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>263</v>
       </c>

</xml_diff>